<commit_message>
Add Papaleguas Digital Menu template (cardapio_papaleguas.html)
</commit_message>
<xml_diff>
--- a/leads_psicologo_sao_paulo.xlsx
+++ b/leads_psicologo_sao_paulo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Elaine Ferreira Psicloga Clnica, Psicolo</t>
+          <t>Psicologo Felipe Faccioli</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Elaine ferreira psicóloga clínica, psicologo...</t>
+          <t>Psicologo felipe faccioli - CNPJ 63.510.039/0001-79</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bairro: Freguesia do Ó. Cidade: São Paulo. Estado: SP.Dom: Fechado. Site elaine-ferreira-psicologa-c...</t>
+          <t>Consulte o CNPJ 63.510.039/0001-79 da empresa PSICOLOGO FELIPE FACCIOLI (FELIPE FACCIOLI DE SOUZA LT...</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -521,28 +521,28 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.terapyas.com.br/sobre/elaine-ferreira-psicologa-clinica-psicologo-atendimento-psicologico-e-terapia-sao-paulo-sp</t>
+          <t>https://cnpj.today/63510039000179</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>(11) 97622-2228</t>
+          <t>(41) 97880-1450</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>5511976222228</t>
+          <t>5541978801450</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Elaine%20Ferreira%20Psicloga%20Clnica%2C%20Psicolo%20sao%20paulo</t>
+          <t>https://www.google.com/maps/search/Psicologo%20felipe%20faccioli%20sao%20paulo</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Elaine Ferreira Psicloga Clnica, Psicolo aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Psicologo felipe faccioli aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -552,29 +552,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Elaine Ferreira Psicloga Clnica, Psicolo?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Psicologo felipe faccioli?</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://wa.me/5511976222228?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Elaine%20Ferreira%20Psicloga%20Clnica%2C%20Psicolo%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541978801450?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Psicologo%20felipe%20faccioli%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://wa.me/5511976222228?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Elaine%20Ferreira%20Psicloga%20Clnica%2C%20Psicolo%3F</t>
+          <t>https://wa.me/5541978801450?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Psicologo%20felipe%20faccioli%3F</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Equilibrio Psicologia Clinica</t>
+          <t>Psiclogo Clnico Particular em Perdizes</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Equilibrio Psicologia Clinica — psicologo em São Paulo/SP</t>
+          <t>Psicólogo Clínico Particular em Perdizes - OneLiv</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>A Equilibrio Psicologia Clinica oferece atendimento com psicólogo em São Paulo/SP, em um espaço acol...</t>
+          <t>"Precisa de ajuda? Explore uma lista completa de psicólogos em Perdizes e encontre o especialista pe...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -599,28 +599,28 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://velora.tech/sp/sao-paulo/psicologo/equilibrio-psicologia-clinica-313048</t>
+          <t>https://oneliv.com.br/psicologo/sao-paulo/perdizes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>(71) 94400-0105</t>
+          <t>(11) 97425-1474</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>5571944000105</t>
+          <t>5511974251474</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Equilibrio%20Psicologia%20Clinica%20sao%20paulo</t>
+          <t>https://www.google.com/maps/search/Psiclogo%20Clnico%20Particular%20em%20Perdizes%20sao%20paulo</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Equilibrio Psicologia Clinica aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Psiclogo Clnico Particular em Perdizes aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -630,29 +630,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Equilibrio Psicologia Clinica?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Psiclogo Clnico Particular em Perdizes?</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://wa.me/5571944000105?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Equilibrio%20Psicologia%20Clinica%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5511974251474?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Psiclogo%20Clnico%20Particular%20em%20Perdizes%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://wa.me/5571944000105?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Equilibrio%20Psicologia%20Clinica%3F</t>
+          <t>https://wa.me/5511974251474?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Psiclogo%20Clnico%20Particular%20em%20Perdizes%3F</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clnica de Psiclogo</t>
+          <t>Terappia</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Clínica de Psicólogo - Agende Sua Sessão - São Paulo - Luana...</t>
+          <t>Terappia - Psicologia Online. Consultas a partir de R$ 40 ...</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -667,38 +667,38 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>De forma geral, a terapia online pode ser útil em praticamente todos os temas que um psicólogo clíni...</t>
+          <t>Terapia online com psicólogos via WhatsApp. Consultas a partir de R$ 40. Encontre o seu psicólogo on...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SITE FORA DO AR (ERRO 404) 🚨</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://psicologaluanaamaral.com.br/psicologo/clinica-de-psicologo-agende-sua-sessao-sao-paulo/</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>(11) 98215-4403</t>
+          <t>(21) 99985-0091</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5511982154403</t>
+          <t>5521999850091</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Clnica%20de%20Psiclogo%20sao%20paulo</t>
+          <t>https://www.google.com/maps/search/Terappia%20sao%20paulo</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Clnica de Psiclogo aí em Sao paulo no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
+Vi o perfil da Terappia aí em Sao paulo no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -708,29 +708,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Clnica de Psiclogo?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Terappia?</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://wa.me/5511982154403?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Clnica%20de%20Psiclogo%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5521999850091?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Terappia%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://wa.me/5511982154403?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Clnica%20de%20Psiclogo%3F</t>
+          <t>https://wa.me/5521999850091?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Terappia%3F</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Somente</t>
+          <t>Clnica de Psicologia em So Paulo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SOMENTE | SAUDE EMOCIONAL</t>
+          <t>Clínica de psicologia em São Paulo - PsicoClinic</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Descomplicamos o acesso à saúde emocional com um canal direto via WhatsApp, onde você pode agendar, ...</t>
+          <t>Com psicóloga em São Paulo referência em tratamentos de excelência, a PsicoClinic é reconhecida pelo...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -755,28 +755,28 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.somente.com.br/</t>
+          <t>https://www.psicoclinic.com.br/</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>(11) 93776-1645</t>
+          <t>(11) 91857-7779</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5511937761645</t>
+          <t>5511918577779</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Somente%20sao%20paulo</t>
+          <t>https://www.google.com/maps/search/Clnica%20de%20psicologia%20em%20So%20Paulo%20sao%20paulo</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Somente aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Clnica de psicologia em So Paulo aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -786,29 +786,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Somente?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Clnica de psicologia em So Paulo?</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://wa.me/5511937761645?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Somente%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5511918577779?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Clnica%20de%20psicologia%20em%20So%20Paulo%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://wa.me/5511937761645?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Somente%3F</t>
+          <t>https://wa.me/5511918577779?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Clnica%20de%20psicologia%20em%20So%20Paulo%3F</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Psicloga Responde Perguntas Sobre Psicol</t>
+          <t>Bem Estar Psicologia</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Psicóloga responde perguntas sobre Psicologia e Psicoterapia</t>
+          <t>Bem Estar Psicologia | Psicólogos e Fonoaudiólogo em São ...</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Cosulta com psicóloga online, neuropsicologo online, psicólogo online preço, psicologos em sao paulo...</t>
+          <t>Clínica de Psicologia e Fonoaudiologia na Zona Norte de São Paulo. Atendimento presencial e online p...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -833,28 +833,28 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.psicologaresponde.com.br/2023/04/psicologa-responde-perguntas-sobre.html</t>
+          <t>https://www.bemestarpsicologia.com.br/</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>(11) 99787-4512</t>
+          <t>(11) 94846-2683</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>5511997874512</t>
+          <t>5511948462683</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Psicloga%20Responde%20Perguntas%20Sobre%20Psicol%20sao%20paulo</t>
+          <t>https://www.google.com/maps/search/Bem%20Estar%20Psicologia%20sao%20paulo</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Psicloga Responde Perguntas Sobre Psicol aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Bem Estar Psicologia aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -864,29 +864,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Psicloga Responde Perguntas Sobre Psicol?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Bem Estar Psicologia?</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://wa.me/5511997874512?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Psicloga%20Responde%20Perguntas%20Sobre%20Psicol%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5511948462683?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Bem%20Estar%20Psicologia%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://wa.me/5511997874512?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Psicloga%20Responde%20Perguntas%20Sobre%20Psicol%3F</t>
+          <t>https://wa.me/5511948462683?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Bem%20Estar%20Psicologia%3F</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Psicloga Terapia de Casal</t>
+          <t>Elaine Ferreira Psicloga Clnica, Psicolo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Psicóloga Terapia de Casal | terapia online | Ana Caroline Pina d</t>
+          <t>Elaine ferreira psicóloga clínica, psicologo...</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -901,38 +901,38 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>As consultas presenciais são apenas em São Paulo. Confira abaixo os consultórios com atendimentos pr...</t>
+          <t>Bairro: Freguesia do Ó. Cidade: São Paulo. Estado: SP.Sua mensagem será enviada para nossa equipe e ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://www.terapyas.com.br/sobre/elaine-ferreira-psicologa-clinica-psicologo-atendimento-psicologico-e-terapia-sao-paulo-sp</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>(11) 95091-1931</t>
+          <t>(11) 97622-2228</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5511950911931</t>
+          <t>5511976222228</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Psicloga%20Terapia%20de%20Casal%20sao%20paulo</t>
+          <t>https://www.google.com/maps/search/Elaine%20ferreira%20psicloga%20clnica%2C%20psicologo...%20sao%20paulo</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Psicloga Terapia de Casal aí em Sao paulo no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Elaine ferreira psicloga clnica, psicologo... aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -942,29 +942,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Psicloga Terapia de Casal?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Elaine ferreira psicloga clnica, psicologo...?</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://wa.me/5511950911931?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Psicloga%20Terapia%20de%20Casal%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5511976222228?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Elaine%20ferreira%20psicloga%20clnica%2C%20psicologo...%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://wa.me/5511950911931?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Psicloga%20Terapia%20de%20Casal%3F</t>
+          <t>https://wa.me/5511976222228?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Elaine%20ferreira%20psicloga%20clnica%2C%20psicologo...%3F</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nossos Contatos</t>
+          <t>Barbearia em So Paulo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nossos contatos | Psicólogos São Paulo</t>
+          <t>Barbearia em São Paulo - perto de mim - Cabeleireiro ...</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Confira aqui todos os nossos contatos. Nosso nosso WhatsApp, e-mail, telefone, chat e endereço admin...</t>
+          <t>Para evitar isso, use os mecanismos de localização do Booksy e encontre os lugares mais próximos da ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -989,28 +989,28 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.psicologossaopaulo.com.br/contato/</t>
+          <t>https://booksy.com/pt-br/s/barbearias/1047773_sao-paulo</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>(11) 98204-5631</t>
+          <t>(11) 94990-8390</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>5511982045631</t>
+          <t>5511949908390</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Nossos%20Contatos%20sao%20paulo</t>
+          <t>https://www.google.com/maps/search/Barbearia%20em%20So%20Paulo%20sao%20paulo</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Nossos Contatos aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia em So Paulo aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1020,95 +1020,17 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Nossos Contatos?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia em So Paulo?</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://wa.me/5511982045631?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Nossos%20Contatos%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5511949908390?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20em%20So%20Paulo%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://wa.me/5511982045631?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Nossos%20Contatos%3F</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Psicloga Sp Maristela Vallim Botari</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Psicóloga SP Maristela Vallim Botari | Terapia Humanizada na Av..</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Sao paulo</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Centro / Região</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Para agendar uma Consulta Acolhimento humanizado Whatsapp Psicóloga (11) 95091-1931. Terapia online ...</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>SITE ATIVO 📱</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>https://www.psicologa-sp.com.br/</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>(11) 95091-1931</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>5511950911931</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/Psicloga%20Sp%20Maristela%20Vallim%20Botari%20sao%20paulo</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Psicloga Sp Maristela Vallim Botari aí em Sao paulo no Google e vi que o site de vocês está um pouco desatualizado para celular.
-Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
-Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
-A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
-Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Psicloga Sp Maristela Vallim Botari?</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>https://wa.me/5511950911931?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Psicloga%20Sp%20Maristela%20Vallim%20Botari%20a%C3%AD%20em%20Sao%20paulo%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>https://wa.me/5511950911931?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Psicloga%20Sp%20Maristela%20Vallim%20Botari%3F</t>
+          <t>https://wa.me/5511949908390?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20em%20So%20Paulo%3F</t>
         </is>
       </c>
     </row>

</xml_diff>